<commit_message>
Version 1.2.0: job orders, QR labels, new header, better pick lists, privacy notice
- Job orders (COH-IDN-F-01, ADM-HIMS-P-03): public request page, JO Log tab
  with ICTU-YYYY-NNNN numbers, priority targets, Part II and III, printed form,
  monthly JO report; the old online form can post to the same log
- QR property labels; scanning one opens a public status page for the unit
- Equipment service and maintenance history (PMs and job orders)
- Header: round seals, no Bagong Pilipinas logo, menu for Refresh and Lock
- Pick lists with add-new at the bottom; picking an employee sets the section
- Data privacy notice (RA 10173) on every page

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdEkDZ9MtY1FWGj4n3zSje
</commit_message>
<xml_diff>
--- a/Register/ICT Inventory and PMS Register (ICTU).xlsx
+++ b/Register/ICT Inventory and PMS Register (ICTU).xlsx
@@ -10,9 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist Results" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JO Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -904,6 +905,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:BA1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="23" customWidth="1" min="22" max="22"/>
+    <col width="24" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="27" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="23" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
+    <col width="21" customWidth="1" min="37" max="37"/>
+    <col width="18" customWidth="1" min="38" max="38"/>
+    <col width="19" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="16" customWidth="1" min="43" max="43"/>
+    <col width="23" customWidth="1" min="44" max="44"/>
+    <col width="15" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="15" customWidth="1" min="49" max="49"/>
+    <col width="16" customWidth="1" min="50" max="50"/>
+    <col width="15" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="14" customWidth="1" min="53" max="53"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date/Time Logged</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>JO No.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Date/Time of Request</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>M.I.</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Section / Unit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Contact / Local No.</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Mode of Request</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment / System</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Brand / Model</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Property / Serial No.</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Urgent?</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Urgent Reason</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Type(s) of Request</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Brief Description</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Section / Unit Head</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Data Privacy Consent</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>ICTU Personnel</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Date/Time Finished</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Findings / Action Taken</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Last Action</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Last Action At</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Print / Share Count</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Action History</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Request ID</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment ID</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Received By</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Date/Time Received</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Date/Time Started</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Mode of Service</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Pulled Out On</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Returned On</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Findings / Cause</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Action Taken</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Parts Used / Needed</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Status Note</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Target Date/Time</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Within Target?</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>CSM Speed</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>CSM Quality</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>CSM Courtesy</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Suggestions</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -952,7 +1289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1289,13 +1626,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1317,7 +1654,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>The records behind the ICT Inventory and PMS app: the equipment masterlist, the PM Log, the checklist answers of each PM and the audit trail.</t>
+          <t>The records behind the ICT Inventory and PMS app: the equipment masterlist, the PM Log, the checklist answers of each PM, the Job Order Log and the audit trail.</t>
         </is>
       </c>
     </row>
@@ -1336,82 +1673,106 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>App version</t>
+          <t>JO form</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>COH-IDN-F-01 Rev. 01, ICTU Job Order Request Form (ADM-HIMS-P-03 ICTU Service Procedure)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>App version</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>One row per unit. Equipment ID (ICT-0001 and up) is given by the app. You may paste new rows here with the ID blank; the app fills it in the next time it opens.</t>
+          <t>1.2.0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>PM Log</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>One row per PM activity. The first 21 columns match ICTU_Preventive_Maintenance_Log.xlsx. PM Ref. No. continues the PM-YYYY-NNN series. Wrong entries are voided, never deleted.</t>
+          <t>One row per unit. Equipment ID (ICT-0001 and up) is given by the app. You may paste new rows here with the ID blank; the app fills it in the next time it opens.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Checklist Results</t>
+          <t>PM Log</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The Done / Issue / N/A answer of every checklist item, by PM Ref. No.</t>
+          <t>One row per PM activity. The first 21 columns match ICTU_Preventive_Maintenance_Log.xlsx. PM Ref. No. continues the PM-YYYY-NNN series. Wrong entries are voided, never deleted.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Lists</t>
+          <t>Checklist Results</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Choices shown in the app. Edit these to add offices, staff, equipment types and their default PM frequency.</t>
+          <t>The Done / Issue / N/A answer of every checklist item, by PM Ref. No.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>PM frequency</t>
+          <t>JO Log</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Monthly, Quarterly, Semi-Annual, Annual, or Not scheduled (checked with its PC) for monitors, keyboards, hubs and other parts of a PC set.</t>
+          <t>One row per job order. The first 33 columns match the old ICTU Job Order Log, so its rows can be pasted here. JO No. is ICTU-YYYY-NNNN. Cancelled job orders stay on record.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Lists</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Choices shown in the app. Edit these to add offices, staff, equipment types and their default PM frequency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PM frequency</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Monthly, Quarterly, Semi-Annual, Annual, or Not scheduled (checked with its PC) for monitors, keyboards, hubs and other parts of a PC set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>Protection</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>After setup, every tab can be edited by hand only by the Sheet owner. The app writes through Apps Script with the ICTU passcode.</t>
         </is>

</xml_diff>

<commit_message>
Version 1.3.0: personal sign-in with roles, monthly backup, CSM link, transfers, stock, TIR, replacement plan, cost per unit, dashboard, incidents, network
- Each ICTU staff member signs in with their own account (Head, Technician, Viewer);
  the old passcode only makes the first Head account. Cleaner sign-in card with the
  privacy notice as a pop-up link.
- Monthly copy of the Sheet to Drive, plus Back up now for the Head.
- Requestor rates the service from a link / QR on the job order once it is closed.
- Transfers and turnovers (PAR / ICS) update the masterlist and print a slip.
- Spare parts and consumables with stock cards; parts issued count toward the unit's cost.
- TIR printed from the job order; replacement plan by age; cost per unit report.
- Dashboard with charts, incident and data breach log, network and IP inventory.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdEkDZ9MtY1FWGj4n3zSje
</commit_message>
<xml_diff>
--- a/Register/ICT Inventory and PMS Register (ICTU).xlsx
+++ b/Register/ICT Inventory and PMS Register (ICTU).xlsx
@@ -11,9 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist Results" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JO Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Movements" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidents" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -605,6 +611,818 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Net ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Name / Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>IP Address</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MAC Address</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VLAN / Subnet</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Brand / Model</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment ID</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Provider / ISP</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Account / Circuit No.</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Bandwidth</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Contract End</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Cost</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>By</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Default PM Frequency</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Office / Section</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ICT Personnel</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Useful Life (years)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Replacement Cost (PHP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Desktop Computer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ABTC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>James Adrian M. Elona</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Head, ICT Unit</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cleaning</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Serviceable</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Accounting Section</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Argie R. Lopez</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Computer Operator II</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Diagnostics</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>For monitoring</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Billing Section</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Counter Reset / Service Mode</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>For repair</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Scanner</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Budget Section</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Software / OS Update</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Unserviceable</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Not scheduled (checked with its PC)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cash Unit</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Virus &amp; Malware Check</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Disposed</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Keyboard / Mouse</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Not scheduled (checked with its PC)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>HRMO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Backup</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>UPS / AVR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Semi-Annual</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ICTU</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Network Check</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Network Device</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Semi-Annual</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Materials Management Unit (MMU)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Hardware Repair / Replacement</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Projector</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Office of the TRC Chief</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Print Test</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Peripheral (USB hub, Wi-Fi dongle, etc.)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Not scheduled (checked with its PC)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ICT Inventory and PMS Register (ICTU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>What this is</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>The records behind the ICT Inventory and PMS app: the equipment masterlist, the PM Log, the checklist answers of each PM, the Job Order Log and the audit trail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PM form</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>COH-IDN-F-02 Rev. 01, ICT Equipment Preventive Maintenance Checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>JO form</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>COH-IDN-F-01 Rev. 01, ICTU Job Order Request Form (ADM-HIMS-P-03 ICTU Service Procedure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>App version</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>One row per unit. Equipment ID (ICT-0001 and up) is given by the app. You may paste new rows here with the ID blank; the app fills it in the next time it opens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>PM Log</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>One row per PM activity. The first 21 columns match ICTU_Preventive_Maintenance_Log.xlsx. PM Ref. No. continues the PM-YYYY-NNN series. Wrong entries are voided, never deleted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Checklist Results</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>The Done / Issue / N/A answer of every checklist item, by PM Ref. No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>JO Log</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>One row per job order. The first 33 columns match the old ICTU Job Order Log, so its rows can be pasted here. JO No. is ICTU-YYYY-NNNN. Cancelled job orders stay on record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ICTU accounts (Head, Technician, Viewer). Passwords are stored only as salted hashes. Manage accounts in the app, not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Transfers and turnovers of equipment (section, end user, accountable officer; PAR / ICS / PTR no.). TR-YYYY-NNN. Never edited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Stock Items / Stock Movements</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Spare parts and consumables, and every receipt, issue and adjustment (SM-YYYY-NNNN). The balance is the sum of the movements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Incidents</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>ICT security incidents and data breaches (INC-YYYY-NNN), with the DPO and NPC dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Network devices, fixed IP addresses and internet lines (NET-NNN). No passwords.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Lists</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Choices shown in the app. Edit these to add offices, staff, equipment types with their default PM frequency, useful life (years) and replacement cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>PM frequency</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Monthly, Quarterly, Semi-Annual, Annual, or Not scheduled (checked with its PC) for monitors, keyboards, hubs and other parts of a PC set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>After setup, every tab can be edited by hand only by the Sheet owner. The app writes through Apps Script, only for a signed-in ICTU account whose role allows it. A copy of the Sheet is saved to Drive every month.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -905,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA1"/>
+  <dimension ref="A1:BG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -961,6 +1779,12 @@
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="16" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
+    <col width="22" customWidth="1" min="57" max="57"/>
+    <col width="25" customWidth="1" min="58" max="58"/>
+    <col width="23" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1227,6 +2051,36 @@
       <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Updated By</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>CSM Token</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>CSM Given At</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>TIR No.</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>TIR Recommendation</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Estimated Repair Cost</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Outside Repair Cost</t>
         </is>
       </c>
     </row>
@@ -1241,46 +2095,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Username</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Full Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>By</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Must Change Password</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Last Sign-in</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
         </is>
       </c>
     </row>
@@ -1295,329 +2179,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Equipment Type</t>
+          <t>Transfer No.</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Default PM Frequency</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Office / Section</t>
+          <t>Equipment ID</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ICT Personnel</t>
+          <t>Kind</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>From Section / Unit</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Maintenance Type</t>
+          <t>From End User</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Condition</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Desktop Computer</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ABTC</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>James Adrian M. Elona</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Head, ICT Unit</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Cleaning</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Serviceable</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Accounting Section</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Argie R. Lopez</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Computer Operator II</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Diagnostics</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>For monitoring</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Printer</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Billing Section</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Counter Reset / Service Mode</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>For repair</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Scanner</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Budget Section</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Software / OS Update</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Unserviceable</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Not scheduled (checked with its PC)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Cash Unit</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Virus &amp; Malware Check</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Disposed</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Keyboard / Mouse</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Not scheduled (checked with its PC)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>HRMO</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Backup</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>UPS / AVR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Semi-Annual</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>ICTU</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Network Check</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Network Device</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Semi-Annual</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Materials Management Unit (MMU)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Hardware Repair / Replacement</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Projector</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Annual</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Office of the TRC Chief</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Print Test</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Peripheral (USB hub, Wi-Fi dongle, etc.)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Not scheduled (checked with its PC)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Procurement</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Annual</t>
+          <t>From Accountable Officer</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>To Section / Unit</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>To End User</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>To Accountable Officer</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PAR / ICS / PTR No.</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Reason / Remarks</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded By</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded At</t>
         </is>
       </c>
     </row>
@@ -1632,149 +2281,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>ICT Inventory and PMS Register (ICTU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>What this is</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>The records behind the ICT Inventory and PMS app: the equipment masterlist, the PM Log, the checklist answers of each PM, the Job Order Log and the audit trail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>PM form</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>COH-IDN-F-02 Rev. 01, ICT Equipment Preventive Maintenance Checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>JO form</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>COH-IDN-F-01 Rev. 01, ICTU Job Order Request Form (ADM-HIMS-P-03 ICTU Service Procedure)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>App version</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>1.2.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>One row per unit. Equipment ID (ICT-0001 and up) is given by the app. You may paste new rows here with the ID blank; the app fills it in the next time it opens.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>PM Log</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>One row per PM activity. The first 21 columns match ICTU_Preventive_Maintenance_Log.xlsx. PM Ref. No. continues the PM-YYYY-NNN series. Wrong entries are voided, never deleted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Checklist Results</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>The Done / Issue / N/A answer of every checklist item, by PM Ref. No.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>JO Log</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>One row per job order. The first 33 columns match the old ICTU Job Order Log, so its rows can be pasted here. JO No. is ICTU-YYYY-NNNN. Cancelled job orders stay on record.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Lists</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Choices shown in the app. Edit these to add offices, staff, equipment types and their default PM frequency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>PM frequency</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Monthly, Quarterly, Semi-Annual, Annual, or Not scheduled (checked with its PC) for monitors, keyboards, hubs and other parts of a PC set.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Protection</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>After setup, every tab can be edited by hand only by the Sheet owner. The app writes through Apps Script with the ICTU passcode.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item Code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reorder Level</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ref No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Item Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Cost</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Reference (JO / PM / PR / IAR)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment ID</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Section / Unit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded By</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded At</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Incident No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Discovered At</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Personal Data Involved?</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Systems / Equipment Affected</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Equipment ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Actions Taken</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Reported to DPO On</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>NPC Notification Needed?</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>NPC Notified On</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Related JO No.</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded By</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Recorded At</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Action History</t>
         </is>
       </c>
     </row>

</xml_diff>